<commit_message>
#3 Poe Injector added in BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Industrial IOT development board-v1.0/BOM/Client-BOM-v1.0.xlsx
+++ b/Design Files/Industrial IOT development board-v1.0/BOM/Client-BOM-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1155" uniqueCount="699">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1163" uniqueCount="701">
   <si>
     <t>#</t>
   </si>
@@ -2116,6 +2116,12 @@
   </si>
   <si>
     <t>18650 battery (x1) - This one is used cell category... New and original not available</t>
+  </si>
+  <si>
+    <t>Omada</t>
+  </si>
+  <si>
+    <t>POE160S</t>
   </si>
 </sst>
 </file>
@@ -2361,9 +2367,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2372,6 +2375,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2661,7 +2667,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L165"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="4" style="4" bestFit="1" customWidth="1"/>
@@ -2685,9 +2691,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -7815,7 +7821,7 @@
       <c r="J161" s="7" t="s">
         <v>693</v>
       </c>
-      <c r="K161" s="18" t="s">
+      <c r="K161" s="17" t="s">
         <v>692</v>
       </c>
     </row>
@@ -7848,7 +7854,7 @@
       <c r="J162" s="9" t="s">
         <v>694</v>
       </c>
-      <c r="K162" s="19" t="s">
+      <c r="K162" s="18" t="s">
         <v>692</v>
       </c>
     </row>
@@ -7881,13 +7887,13 @@
       <c r="J163" s="7">
         <v>1</v>
       </c>
-      <c r="K163" s="18" t="s">
+      <c r="K163" s="17" t="s">
         <v>692</v>
       </c>
     </row>
     <row r="164" spans="2:12" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B164" s="11">
-        <f t="shared" ref="B164" si="1">ROW(B164) - ROW($B$2)</f>
+        <f t="shared" ref="B164:B165" si="1">ROW(B164) - ROW($B$2)</f>
         <v>162</v>
       </c>
       <c r="C164" s="12" t="s">
@@ -7914,11 +7920,44 @@
       <c r="J164" s="9">
         <v>1</v>
       </c>
-      <c r="K164" s="19" t="s">
+      <c r="K164" s="18" t="s">
         <v>692</v>
       </c>
-      <c r="L164" s="20" t="s">
+      <c r="L164" s="19" t="s">
         <v>698</v>
+      </c>
+    </row>
+    <row r="165" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B165" s="11">
+        <f t="shared" si="1"/>
+        <v>163</v>
+      </c>
+      <c r="C165" s="12" t="s">
+        <v>690</v>
+      </c>
+      <c r="D165" s="9" t="s">
+        <v>688</v>
+      </c>
+      <c r="E165" s="10" t="s">
+        <v>688</v>
+      </c>
+      <c r="F165" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="G165" s="8" t="s">
+        <v>700</v>
+      </c>
+      <c r="H165" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="I165" s="8" t="s">
+        <v>688</v>
+      </c>
+      <c r="J165" s="9">
+        <v>1</v>
+      </c>
+      <c r="K165" s="18" t="s">
+        <v>699</v>
       </c>
     </row>
   </sheetData>
@@ -7930,8 +7969,9 @@
     <hyperlink ref="K162" r:id="rId2"/>
     <hyperlink ref="K163" r:id="rId3"/>
     <hyperlink ref="K164" r:id="rId4"/>
+    <hyperlink ref="K165" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>